<commit_message>
Expand battle GAS with cues, melee sweep, and wave AI.
Luban now drives damage types and cue tables, GamePlay adds slot-based agents, and the Battle scene presents cues instead of only logging casts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/battle/effect.xlsx
+++ b/Config/Luban/Datas/battle/effect.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="effect" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,71 @@
           <t>mod_magnitude</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>granted_tags</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>required_tags</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>blocked_tags</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>immunity_tags</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>period</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>max_stacks</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>cost_attribute</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>cost_amount</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>execution_type</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>execution_effect_id</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>cue_apply</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>cue_remove</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>shield_value</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -471,7 +536,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>EffectDurationType</t>
+          <t>CfgEffectDurationType</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -481,7 +546,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>EffectStackingType</t>
+          <t>CfgEffectStackingType</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,6 +560,71 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>CfgEffectExecutionType</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -537,6 +667,71 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
         <is>
           <t>c</t>
         </is>
@@ -546,28 +741,451 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Buff.AttackUp</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+          <t>Stun</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>State.CrowdControl.Stunned,Effect.Debuff</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Cue.Stun</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Cue.Stun</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Poison</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>StackCount</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Effect.Debuff</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>2</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Damage</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Cue.Poison</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Cue.Poison</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ShieldBubble</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>RefreshDuration</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Effect.Buff</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Cue.Shield</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Cue.Shield</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Vulnerable</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>RefreshDuration</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>IncomingDamageMultiplier</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
         <v>1</v>
       </c>
-      <c r="D4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Attack</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>5</v>
+      <c r="H7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Effect.Debuff</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Cue.Vulnerable</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Cue.Vulnerable</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ComboWindow</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>RefreshDuration</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Ability.Melee.ComboWindow</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IFrame</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>RefreshDuration</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Immunity.Damage,State.Dodging</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Cue.Dodge.Cast</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Cue.Dodge.Cast</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Knockdown</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>State.CrowdControl.KnockedDown,Effect.Debuff</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Cue.Knockdown</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Cue.Knockdown</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>